<commit_message>
Add mini case study for combined heat resilience constriang dev
</commit_message>
<xml_diff>
--- a/data/example-selfsufficiency/Global_Parameters.xlsx
+++ b/data/example-selfsufficiency/Global_Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon Malacek\Code\LEGO-Pyomo\data\example-selfsufficiency\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8B4A51-2FCF-4369-89E6-503502C9FE04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EFA191E-0B9A-4AF5-AD0F-1D76B9D607BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="28920" windowHeight="17400" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Parameters" sheetId="121" r:id="rId1"/>
@@ -452,21 +452,7 @@
     <cellStyle name="Standard 3" xfId="6" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
     <cellStyle name="Standard 4" xfId="7" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF4E9C49"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFB90135"/>
-      </font>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <font>
         <b/>
@@ -1134,7 +1120,7 @@
         <v>47</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>48</v>
@@ -1151,7 +1137,7 @@
         <v>43</v>
       </c>
       <c r="C25" s="9">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>45</v>
@@ -1168,54 +1154,46 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C5">
-    <cfRule type="cellIs" dxfId="13" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="21" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="22" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8">
-    <cfRule type="cellIs" dxfId="11" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="23" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="24" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C12">
-    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="10" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15">
-    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="8" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19">
-    <cfRule type="cellIs" dxfId="5" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="15" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="16" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C25">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
+  <conditionalFormatting sqref="C24:C25">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1238,21 +1216,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004934E3CB1C58BA43BC6E229E2BF20201" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e33ccc94e63df24f58cb47229b46e190">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87003a75-b64f-4b22-bf19-aa30740e3d46" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f0f7a5bb162b669de9ce8ff8278c29f" ns2:_="">
     <xsd:import namespace="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
@@ -1398,31 +1361,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{773946F7-566C-458F-95C9-79B0CCE20E87}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1438,4 +1392,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>